<commit_message>
Sépare les deux approches de traduction sur des champs distincts et documente les résultats
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> ecd2e651b28ec34d85e07218d879e57c554515c1
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-ANSPatient.xlsx
+++ b/main/ig/StructureDefinition-ANSPatient.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="128">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-27T15:37:21+00:00</t>
+    <t>2026-03-27T15:45:43+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -82,7 +82,7 @@
   </si>
   <si>
     <t>Extension du modèle EHDSPatient pour le contexte français.
-Traduit en français les libellés des éléments hérités et ajoute des champs spécifiques au système de santé français.</t>
+Traduit en français les libellés des éléments hérités (deux approches testées) et ajoute des champs spécifiques au système de santé français.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -264,10 +264,7 @@
 </t>
   </si>
   <si>
-    <t>Identifiant du patient</t>
-  </si>
-  <si>
-    <t>Identifiant unique du patient dans un périmètre défini (par ex. identifiant national de santé, ou identifiant temporaire du DPI).</t>
+    <t>An identifier of the patient that is unique within a defined scope (typically a national patient identifier, but it can also be a temporary identifier issued by the EHR).</t>
   </si>
   <si>
     <t>EHDSPatient.identifier</t>
@@ -312,10 +309,7 @@
 dateTime</t>
   </si>
   <si>
-    <t>Patient décédé / Date de décès</t>
-  </si>
-  <si>
-    <t>Indique si le patient est décédé ou renseigne la date de décès.</t>
+    <t>Whether the patient is deceased or date of death.</t>
   </si>
   <si>
     <t>EHDSPatient.deceased[x]</t>
@@ -350,10 +344,7 @@
 </t>
   </si>
   <si>
-    <t>Adresse(s)</t>
-  </si>
-  <si>
-    <t>Adresses postale et personnelle/professionnelle du patient.</t>
+    <t>The addresses are always sequences of address parts (e.g. street address line, country, postal code, city) even if postal address formats may vary depending on the country. An address may or may not include a specific use code; if this attribute is not present it is assumed to be the default address useful for any purpose.</t>
   </si>
   <si>
     <t>EHDSPatient.address</t>
@@ -366,10 +357,7 @@
 </t>
   </si>
   <si>
-    <t>Coordonnées de contact</t>
-  </si>
-  <si>
-    <t>Informations de contact du patient (téléphone, email, etc.).</t>
+    <t>Contact information.</t>
   </si>
   <si>
     <t>EHDSPatient.telecom</t>
@@ -1007,11 +995,9 @@
       <c r="K3" t="s" s="2">
         <v>81</v>
       </c>
-      <c r="L3" t="s" s="2">
+      <c r="L3" s="2"/>
+      <c r="M3" t="s" s="2">
         <v>82</v>
-      </c>
-      <c r="M3" t="s" s="2">
-        <v>83</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -1062,7 +1048,7 @@
         <v>73</v>
       </c>
       <c r="AF3" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AG3" t="s" s="2">
         <v>80</v>
@@ -1082,10 +1068,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" t="s" s="2">
@@ -1108,13 +1094,13 @@
         <v>73</v>
       </c>
       <c r="K4" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="L4" t="s" s="2">
         <v>86</v>
       </c>
-      <c r="L4" t="s" s="2">
+      <c r="M4" t="s" s="2">
         <v>87</v>
-      </c>
-      <c r="M4" t="s" s="2">
-        <v>88</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -1165,7 +1151,7 @@
         <v>73</v>
       </c>
       <c r="AF4" t="s" s="2">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AG4" t="s" s="2">
         <v>74</v>
@@ -1185,10 +1171,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B5" t="s" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" t="s" s="2">
@@ -1211,13 +1197,13 @@
         <v>73</v>
       </c>
       <c r="K5" t="s" s="2">
+        <v>90</v>
+      </c>
+      <c r="L5" t="s" s="2">
         <v>91</v>
       </c>
-      <c r="L5" t="s" s="2">
+      <c r="M5" t="s" s="2">
         <v>92</v>
-      </c>
-      <c r="M5" t="s" s="2">
-        <v>93</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1268,7 +1254,7 @@
         <v>73</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>74</v>
@@ -1288,10 +1274,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1314,13 +1300,13 @@
         <v>73</v>
       </c>
       <c r="K6" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="L6" t="s" s="2">
         <v>96</v>
       </c>
-      <c r="L6" t="s" s="2">
-        <v>97</v>
-      </c>
       <c r="M6" t="s" s="2">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -1371,7 +1357,7 @@
         <v>73</v>
       </c>
       <c r="AF6" t="s" s="2">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="AG6" t="s" s="2">
         <v>74</v>
@@ -1391,10 +1377,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1417,13 +1403,13 @@
         <v>73</v>
       </c>
       <c r="K7" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="L7" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="M7" t="s" s="2">
         <v>101</v>
-      </c>
-      <c r="L7" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="M7" t="s" s="2">
-        <v>103</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1450,31 +1436,31 @@
         <v>73</v>
       </c>
       <c r="X7" t="s" s="2">
+        <v>102</v>
+      </c>
+      <c r="Y7" t="s" s="2">
+        <v>103</v>
+      </c>
+      <c r="Z7" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AA7" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AB7" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AC7" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AD7" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AE7" t="s" s="2">
+        <v>73</v>
+      </c>
+      <c r="AF7" t="s" s="2">
         <v>104</v>
-      </c>
-      <c r="Y7" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="Z7" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AA7" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AB7" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AC7" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AD7" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AE7" t="s" s="2">
-        <v>73</v>
-      </c>
-      <c r="AF7" t="s" s="2">
-        <v>106</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>74</v>
@@ -1494,10 +1480,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1520,13 +1506,11 @@
         <v>73</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>108</v>
-      </c>
-      <c r="L8" t="s" s="2">
-        <v>109</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="L8" s="2"/>
       <c r="M8" t="s" s="2">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -1577,7 +1561,7 @@
         <v>73</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>74</v>
@@ -1597,10 +1581,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1623,13 +1607,11 @@
         <v>73</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="L9" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="L9" s="2"/>
       <c r="M9" t="s" s="2">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1680,7 +1662,7 @@
         <v>73</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>74</v>
@@ -1700,10 +1682,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
@@ -1729,10 +1711,10 @@
         <v>81</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1783,7 +1765,7 @@
         <v>73</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>74</v>
@@ -1803,10 +1785,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -1832,10 +1814,10 @@
         <v>81</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -1886,7 +1868,7 @@
         <v>73</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>74</v>
@@ -1906,10 +1888,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -1932,13 +1914,13 @@
         <v>73</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -1989,7 +1971,7 @@
         <v>73</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>74</v>
@@ -2009,10 +1991,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2035,13 +2017,13 @@
         <v>73</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -2092,7 +2074,7 @@
         <v>73</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>74</v>
@@ -2112,10 +2094,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2138,13 +2120,13 @@
         <v>73</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2195,7 +2177,7 @@
         <v>73</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>74</v>

</xml_diff>